<commit_message>
chore: ARCONEL update — data through Aug 2026
</commit_message>
<xml_diff>
--- a/electricidad/facturacion_clientes_regulados_resumen.xlsx
+++ b/electricidad/facturacion_clientes_regulados_resumen.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,7 +796,7 @@
         <v>2158.8</v>
       </c>
       <c r="C2" t="n">
-        <v>1963.3</v>
+        <v>1957.9</v>
       </c>
     </row>
     <row r="3">
@@ -809,7 +809,7 @@
         <v>1848.8</v>
       </c>
       <c r="C3" t="n">
-        <v>1971.2</v>
+        <v>1965.9</v>
       </c>
     </row>
     <row r="4">
@@ -822,7 +822,7 @@
         <v>2078.4</v>
       </c>
       <c r="C4" t="n">
-        <v>1979</v>
+        <v>1973.8</v>
       </c>
     </row>
     <row r="5">
@@ -835,7 +835,7 @@
         <v>2072.8</v>
       </c>
       <c r="C5" t="n">
-        <v>1986.8</v>
+        <v>1981.8</v>
       </c>
     </row>
     <row r="6">
@@ -848,7 +848,7 @@
         <v>2090.8</v>
       </c>
       <c r="C6" t="n">
-        <v>1994.6</v>
+        <v>1989.8</v>
       </c>
     </row>
     <row r="7">
@@ -861,7 +861,7 @@
         <v>1920.9</v>
       </c>
       <c r="C7" t="n">
-        <v>2002.4</v>
+        <v>1997.8</v>
       </c>
     </row>
     <row r="8">
@@ -874,7 +874,7 @@
         <v>1935.5</v>
       </c>
       <c r="C8" t="n">
-        <v>2010.3</v>
+        <v>2005.8</v>
       </c>
     </row>
     <row r="9">
@@ -887,7 +887,7 @@
         <v>1954.2</v>
       </c>
       <c r="C9" t="n">
-        <v>2018.1</v>
+        <v>2013.8</v>
       </c>
     </row>
     <row r="10">
@@ -900,7 +900,7 @@
         <v>1936.6</v>
       </c>
       <c r="C10" t="n">
-        <v>2025.9</v>
+        <v>2021.7</v>
       </c>
     </row>
     <row r="11">
@@ -913,7 +913,7 @@
         <v>1978.1</v>
       </c>
       <c r="C11" t="n">
-        <v>2033.7</v>
+        <v>2029.7</v>
       </c>
     </row>
     <row r="12">
@@ -926,7 +926,7 @@
         <v>1962.9</v>
       </c>
       <c r="C12" t="n">
-        <v>2041.6</v>
+        <v>2037.7</v>
       </c>
     </row>
     <row r="13">
@@ -939,7 +939,7 @@
         <v>2065.3</v>
       </c>
       <c r="C13" t="n">
-        <v>2049.4</v>
+        <v>2045.7</v>
       </c>
     </row>
     <row r="14">
@@ -952,7 +952,7 @@
         <v>2214.6</v>
       </c>
       <c r="C14" t="n">
-        <v>2057.2</v>
+        <v>2053.7</v>
       </c>
     </row>
     <row r="15">
@@ -965,7 +965,7 @@
         <v>2146.8</v>
       </c>
       <c r="C15" t="n">
-        <v>2065</v>
+        <v>2061.7</v>
       </c>
     </row>
     <row r="16">
@@ -978,7 +978,7 @@
         <v>2357</v>
       </c>
       <c r="C16" t="n">
-        <v>2072.8</v>
+        <v>2069.6</v>
       </c>
     </row>
     <row r="17">
@@ -991,7 +991,7 @@
         <v>2274.1</v>
       </c>
       <c r="C17" t="n">
-        <v>2080.7</v>
+        <v>2077.6</v>
       </c>
     </row>
     <row r="18">
@@ -1004,7 +1004,7 @@
         <v>2330.3</v>
       </c>
       <c r="C18" t="n">
-        <v>2088.5</v>
+        <v>2085.6</v>
       </c>
     </row>
     <row r="19">
@@ -1017,7 +1017,7 @@
         <v>2179.6</v>
       </c>
       <c r="C19" t="n">
-        <v>2096.3</v>
+        <v>2093.6</v>
       </c>
     </row>
     <row r="20">
@@ -1030,7 +1030,7 @@
         <v>2160.9</v>
       </c>
       <c r="C20" t="n">
-        <v>2104.1</v>
+        <v>2101.6</v>
       </c>
     </row>
     <row r="21">
@@ -1043,7 +1043,7 @@
         <v>2195.7</v>
       </c>
       <c r="C21" t="n">
-        <v>2112</v>
+        <v>2109.6</v>
       </c>
     </row>
     <row r="22">
@@ -1056,7 +1056,7 @@
         <v>2112.2</v>
       </c>
       <c r="C22" t="n">
-        <v>2119.8</v>
+        <v>2117.5</v>
       </c>
     </row>
     <row r="23">
@@ -1069,7 +1069,7 @@
         <v>2101.2</v>
       </c>
       <c r="C23" t="n">
-        <v>2127.6</v>
+        <v>2125.5</v>
       </c>
     </row>
     <row r="24">
@@ -1082,7 +1082,7 @@
         <v>2202.4</v>
       </c>
       <c r="C24" t="n">
-        <v>2135.4</v>
+        <v>2133.5</v>
       </c>
     </row>
     <row r="25">
@@ -1095,7 +1095,7 @@
         <v>2303.2</v>
       </c>
       <c r="C25" t="n">
-        <v>2143.3</v>
+        <v>2141.5</v>
       </c>
     </row>
     <row r="26">
@@ -1108,7 +1108,7 @@
         <v>2415.8</v>
       </c>
       <c r="C26" t="n">
-        <v>2151.1</v>
+        <v>2149.5</v>
       </c>
     </row>
     <row r="27">
@@ -1121,7 +1121,7 @@
         <v>2259.1</v>
       </c>
       <c r="C27" t="n">
-        <v>2158.9</v>
+        <v>2157.5</v>
       </c>
     </row>
     <row r="28">
@@ -1134,7 +1134,7 @@
         <v>2183.1</v>
       </c>
       <c r="C28" t="n">
-        <v>2166.7</v>
+        <v>2165.4</v>
       </c>
     </row>
     <row r="29">
@@ -1147,7 +1147,7 @@
         <v>2026.2</v>
       </c>
       <c r="C29" t="n">
-        <v>2174.5</v>
+        <v>2173.4</v>
       </c>
     </row>
     <row r="30">
@@ -1160,7 +1160,7 @@
         <v>2190.4</v>
       </c>
       <c r="C30" t="n">
-        <v>2182.4</v>
+        <v>2181.4</v>
       </c>
     </row>
     <row r="31">
@@ -1173,7 +1173,7 @@
         <v>2185.5</v>
       </c>
       <c r="C31" t="n">
-        <v>2190.2</v>
+        <v>2189.4</v>
       </c>
     </row>
     <row r="32">
@@ -1186,7 +1186,7 @@
         <v>2207.7</v>
       </c>
       <c r="C32" t="n">
-        <v>2198</v>
+        <v>2197.4</v>
       </c>
     </row>
     <row r="33">
@@ -1199,7 +1199,7 @@
         <v>2147.2</v>
       </c>
       <c r="C33" t="n">
-        <v>2205.8</v>
+        <v>2205.4</v>
       </c>
     </row>
     <row r="34">
@@ -1212,7 +1212,7 @@
         <v>2051.3</v>
       </c>
       <c r="C34" t="n">
-        <v>2213.7</v>
+        <v>2213.3</v>
       </c>
     </row>
     <row r="35">
@@ -1225,7 +1225,7 @@
         <v>2182.6</v>
       </c>
       <c r="C35" t="n">
-        <v>2221.5</v>
+        <v>2221.3</v>
       </c>
     </row>
     <row r="36">
@@ -1251,7 +1251,7 @@
         <v>2276.4</v>
       </c>
       <c r="C37" t="n">
-        <v>2237.1</v>
+        <v>2237.3</v>
       </c>
     </row>
     <row r="38">
@@ -1264,7 +1264,7 @@
         <v>2175.8</v>
       </c>
       <c r="C38" t="n">
-        <v>2244.9</v>
+        <v>2245.3</v>
       </c>
     </row>
     <row r="39">
@@ -1277,7 +1277,7 @@
         <v>2028.4</v>
       </c>
       <c r="C39" t="n">
-        <v>2252.8</v>
+        <v>2253.3</v>
       </c>
     </row>
     <row r="40">
@@ -1290,7 +1290,7 @@
         <v>2448.4</v>
       </c>
       <c r="C40" t="n">
-        <v>2260.6</v>
+        <v>2261.2</v>
       </c>
     </row>
     <row r="41">
@@ -1303,7 +1303,7 @@
         <v>2375.5</v>
       </c>
       <c r="C41" t="n">
-        <v>2268.4</v>
+        <v>2269.2</v>
       </c>
     </row>
     <row r="42">
@@ -1316,7 +1316,7 @@
         <v>2203.9</v>
       </c>
       <c r="C42" t="n">
-        <v>2276.2</v>
+        <v>2277.2</v>
       </c>
     </row>
     <row r="43">
@@ -1329,7 +1329,7 @@
         <v>2076.6</v>
       </c>
       <c r="C43" t="n">
-        <v>2284.1</v>
+        <v>2285.2</v>
       </c>
     </row>
     <row r="44">
@@ -1342,7 +1342,7 @@
         <v>2123.1</v>
       </c>
       <c r="C44" t="n">
-        <v>2291.9</v>
+        <v>2293.2</v>
       </c>
     </row>
     <row r="45">
@@ -1355,7 +1355,7 @@
         <v>2156.9</v>
       </c>
       <c r="C45" t="n">
-        <v>2299.7</v>
+        <v>2301.2</v>
       </c>
     </row>
     <row r="46">
@@ -1368,7 +1368,7 @@
         <v>2128</v>
       </c>
       <c r="C46" t="n">
-        <v>2307.5</v>
+        <v>2309.1</v>
       </c>
     </row>
     <row r="47">
@@ -1381,7 +1381,7 @@
         <v>2245.8</v>
       </c>
       <c r="C47" t="n">
-        <v>2315.4</v>
+        <v>2317.1</v>
       </c>
     </row>
     <row r="48">
@@ -1394,7 +1394,7 @@
         <v>2163</v>
       </c>
       <c r="C48" t="n">
-        <v>2323.2</v>
+        <v>2325.1</v>
       </c>
     </row>
     <row r="49">
@@ -1407,7 +1407,7 @@
         <v>2373.7</v>
       </c>
       <c r="C49" t="n">
-        <v>2331</v>
+        <v>2333.1</v>
       </c>
     </row>
     <row r="50">
@@ -1420,7 +1420,7 @@
         <v>2296.2</v>
       </c>
       <c r="C50" t="n">
-        <v>2338.8</v>
+        <v>2341.1</v>
       </c>
     </row>
     <row r="51">
@@ -1433,7 +1433,7 @@
         <v>2085.2</v>
       </c>
       <c r="C51" t="n">
-        <v>2346.6</v>
+        <v>2349.1</v>
       </c>
     </row>
     <row r="52">
@@ -1446,7 +1446,7 @@
         <v>2439</v>
       </c>
       <c r="C52" t="n">
-        <v>2354.5</v>
+        <v>2357</v>
       </c>
     </row>
     <row r="53">
@@ -1459,7 +1459,7 @@
         <v>2386.6</v>
       </c>
       <c r="C53" t="n">
-        <v>2362.3</v>
+        <v>2365</v>
       </c>
     </row>
     <row r="54">
@@ -1472,7 +1472,7 @@
         <v>2369.3</v>
       </c>
       <c r="C54" t="n">
-        <v>2370.1</v>
+        <v>2373</v>
       </c>
     </row>
     <row r="55">
@@ -1485,7 +1485,7 @@
         <v>2119</v>
       </c>
       <c r="C55" t="n">
-        <v>2377.9</v>
+        <v>2381</v>
       </c>
     </row>
     <row r="56">
@@ -1498,7 +1498,7 @@
         <v>2230.9</v>
       </c>
       <c r="C56" t="n">
-        <v>2385.8</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="57">
@@ -1511,7 +1511,7 @@
         <v>2246.6</v>
       </c>
       <c r="C57" t="n">
-        <v>2393.6</v>
+        <v>2397</v>
       </c>
     </row>
     <row r="58">
@@ -1524,7 +1524,7 @@
         <v>2258.1</v>
       </c>
       <c r="C58" t="n">
-        <v>2401.4</v>
+        <v>2404.9</v>
       </c>
     </row>
     <row r="59">
@@ -1537,7 +1537,7 @@
         <v>2272.8</v>
       </c>
       <c r="C59" t="n">
-        <v>2409.2</v>
+        <v>2412.9</v>
       </c>
     </row>
     <row r="60">
@@ -1550,7 +1550,7 @@
         <v>2267.5</v>
       </c>
       <c r="C60" t="n">
-        <v>2417</v>
+        <v>2420.9</v>
       </c>
     </row>
     <row r="61">
@@ -1563,7 +1563,7 @@
         <v>2481.9</v>
       </c>
       <c r="C61" t="n">
-        <v>2424.9</v>
+        <v>2428.9</v>
       </c>
     </row>
     <row r="62">
@@ -1576,7 +1576,7 @@
         <v>2582</v>
       </c>
       <c r="C62" t="n">
-        <v>2432.7</v>
+        <v>2436.9</v>
       </c>
     </row>
     <row r="63">
@@ -1589,7 +1589,7 @@
         <v>2245</v>
       </c>
       <c r="C63" t="n">
-        <v>2440.5</v>
+        <v>2444.9</v>
       </c>
     </row>
     <row r="64">
@@ -1602,7 +1602,7 @@
         <v>2543.7</v>
       </c>
       <c r="C64" t="n">
-        <v>2448.3</v>
+        <v>2452.8</v>
       </c>
     </row>
     <row r="65">
@@ -1615,7 +1615,7 @@
         <v>2492.6</v>
       </c>
       <c r="C65" t="n">
-        <v>2456.2</v>
+        <v>2460.8</v>
       </c>
     </row>
     <row r="66">
@@ -1628,7 +1628,7 @@
         <v>2769.1</v>
       </c>
       <c r="C66" t="n">
-        <v>2464</v>
+        <v>2468.8</v>
       </c>
     </row>
     <row r="67">
@@ -1641,7 +1641,7 @@
         <v>2643.2</v>
       </c>
       <c r="C67" t="n">
-        <v>2471.8</v>
+        <v>2476.8</v>
       </c>
     </row>
     <row r="68">
@@ -1654,7 +1654,7 @@
         <v>2716.3</v>
       </c>
       <c r="C68" t="n">
-        <v>2479.6</v>
+        <v>2484.8</v>
       </c>
     </row>
     <row r="69">
@@ -1667,7 +1667,7 @@
         <v>2555.7</v>
       </c>
       <c r="C69" t="n">
-        <v>2487.5</v>
+        <v>2492.8</v>
       </c>
     </row>
     <row r="70">
@@ -1680,7 +1680,7 @@
         <v>2489.4</v>
       </c>
       <c r="C70" t="n">
-        <v>2495.3</v>
+        <v>2500.7</v>
       </c>
     </row>
     <row r="71">
@@ -1693,7 +1693,7 @@
         <v>2585.2</v>
       </c>
       <c r="C71" t="n">
-        <v>2503.1</v>
+        <v>2508.7</v>
       </c>
     </row>
     <row r="72">
@@ -1706,7 +1706,7 @@
         <v>2403.3</v>
       </c>
       <c r="C72" t="n">
-        <v>2510.9</v>
+        <v>2516.7</v>
       </c>
     </row>
     <row r="73">
@@ -1719,7 +1719,7 @@
         <v>2513.7</v>
       </c>
       <c r="C73" t="n">
-        <v>2518.7</v>
+        <v>2524.7</v>
       </c>
     </row>
     <row r="74">
@@ -1732,7 +1732,7 @@
         <v>2615.5</v>
       </c>
       <c r="C74" t="n">
-        <v>2526.6</v>
+        <v>2532.7</v>
       </c>
     </row>
     <row r="75">
@@ -1745,7 +1745,7 @@
         <v>2487.6</v>
       </c>
       <c r="C75" t="n">
-        <v>2534.4</v>
+        <v>2540.7</v>
       </c>
     </row>
     <row r="76">
@@ -1758,7 +1758,7 @@
         <v>2757.3</v>
       </c>
       <c r="C76" t="n">
-        <v>2542.2</v>
+        <v>2548.6</v>
       </c>
     </row>
     <row r="77">
@@ -1771,7 +1771,7 @@
         <v>2556.3</v>
       </c>
       <c r="C77" t="n">
-        <v>2550</v>
+        <v>2556.6</v>
       </c>
     </row>
     <row r="78">
@@ -1784,7 +1784,7 @@
         <v>2708.4</v>
       </c>
       <c r="C78" t="n">
-        <v>2557.9</v>
+        <v>2564.6</v>
       </c>
     </row>
     <row r="79">
@@ -1797,7 +1797,7 @@
         <v>2518.3</v>
       </c>
       <c r="C79" t="n">
-        <v>2565.7</v>
+        <v>2572.6</v>
       </c>
     </row>
     <row r="80">
@@ -1810,7 +1810,7 @@
         <v>2537</v>
       </c>
       <c r="C80" t="n">
-        <v>2573.5</v>
+        <v>2580.6</v>
       </c>
     </row>
     <row r="81">
@@ -1823,7 +1823,7 @@
         <v>2514.8</v>
       </c>
       <c r="C81" t="n">
-        <v>2581.3</v>
+        <v>2588.6</v>
       </c>
     </row>
     <row r="82">
@@ -1836,7 +1836,7 @@
         <v>2286.8</v>
       </c>
       <c r="C82" t="n">
-        <v>2589.1</v>
+        <v>2596.5</v>
       </c>
     </row>
     <row r="83">
@@ -1849,7 +1849,7 @@
         <v>1975.5</v>
       </c>
       <c r="C83" t="n">
-        <v>2597</v>
+        <v>2604.5</v>
       </c>
     </row>
     <row r="84">
@@ -1862,7 +1862,7 @@
         <v>1853.5</v>
       </c>
       <c r="C84" t="n">
-        <v>2604.8</v>
+        <v>2612.5</v>
       </c>
     </row>
     <row r="85">
@@ -1875,7 +1875,7 @@
         <v>2355.2</v>
       </c>
       <c r="C85" t="n">
-        <v>2612.6</v>
+        <v>2620.5</v>
       </c>
     </row>
     <row r="86">
@@ -1888,7 +1888,7 @@
         <v>2604.6</v>
       </c>
       <c r="C86" t="n">
-        <v>2620.4</v>
+        <v>2628.5</v>
       </c>
     </row>
     <row r="87">
@@ -1901,7 +1901,7 @@
         <v>2566.3</v>
       </c>
       <c r="C87" t="n">
-        <v>2628.3</v>
+        <v>2636.5</v>
       </c>
     </row>
     <row r="88">
@@ -1914,7 +1914,7 @@
         <v>2849</v>
       </c>
       <c r="C88" t="n">
-        <v>2636.1</v>
+        <v>2644.4</v>
       </c>
     </row>
     <row r="89">
@@ -1927,7 +1927,7 @@
         <v>2774.5</v>
       </c>
       <c r="C89" t="n">
-        <v>2643.9</v>
+        <v>2652.4</v>
       </c>
     </row>
     <row r="90">
@@ -1940,7 +1940,7 @@
         <v>2794.3</v>
       </c>
       <c r="C90" t="n">
-        <v>2651.7</v>
+        <v>2660.4</v>
       </c>
     </row>
     <row r="91">
@@ -1953,7 +1953,7 @@
         <v>2573.7</v>
       </c>
       <c r="C91" t="n">
-        <v>2659.6</v>
+        <v>2668.4</v>
       </c>
     </row>
     <row r="92">
@@ -1966,7 +1966,7 @@
         <v>2605.6</v>
       </c>
       <c r="C92" t="n">
-        <v>2667.4</v>
+        <v>2676.4</v>
       </c>
     </row>
     <row r="93">
@@ -1979,7 +1979,7 @@
         <v>2592.2</v>
       </c>
       <c r="C93" t="n">
-        <v>2675.2</v>
+        <v>2684.4</v>
       </c>
     </row>
     <row r="94">
@@ -1992,7 +1992,7 @@
         <v>2667.9</v>
       </c>
       <c r="C94" t="n">
-        <v>2683</v>
+        <v>2692.3</v>
       </c>
     </row>
     <row r="95">
@@ -2005,7 +2005,7 @@
         <v>2802.6</v>
       </c>
       <c r="C95" t="n">
-        <v>2690.8</v>
+        <v>2700.3</v>
       </c>
     </row>
     <row r="96">
@@ -2018,7 +2018,7 @@
         <v>2696.6</v>
       </c>
       <c r="C96" t="n">
-        <v>2698.7</v>
+        <v>2708.3</v>
       </c>
     </row>
     <row r="97">
@@ -2031,7 +2031,7 @@
         <v>2828.5</v>
       </c>
       <c r="C97" t="n">
-        <v>2706.5</v>
+        <v>2716.3</v>
       </c>
     </row>
     <row r="98">
@@ -2044,7 +2044,7 @@
         <v>2685.6</v>
       </c>
       <c r="C98" t="n">
-        <v>2714.3</v>
+        <v>2724.3</v>
       </c>
     </row>
     <row r="99">
@@ -2057,7 +2057,7 @@
         <v>2609.1</v>
       </c>
       <c r="C99" t="n">
-        <v>2722.1</v>
+        <v>2732.3</v>
       </c>
     </row>
     <row r="100">
@@ -2070,7 +2070,7 @@
         <v>3010.2</v>
       </c>
       <c r="C100" t="n">
-        <v>2730</v>
+        <v>2740.2</v>
       </c>
     </row>
     <row r="101">
@@ -2083,7 +2083,7 @@
         <v>2911.6</v>
       </c>
       <c r="C101" t="n">
-        <v>2737.8</v>
+        <v>2748.2</v>
       </c>
     </row>
     <row r="102">
@@ -2096,7 +2096,7 @@
         <v>3074.6</v>
       </c>
       <c r="C102" t="n">
-        <v>2745.6</v>
+        <v>2756.2</v>
       </c>
     </row>
     <row r="103">
@@ -2109,7 +2109,7 @@
         <v>3040.6</v>
       </c>
       <c r="C103" t="n">
-        <v>2753.4</v>
+        <v>2764.2</v>
       </c>
     </row>
     <row r="104">
@@ -2119,10 +2119,23 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>3205.9</v>
+        <v>3208.7</v>
       </c>
       <c r="C104" t="n">
-        <v>2761.2</v>
+        <v>2772.2</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>3058.6</v>
+      </c>
+      <c r="C105" t="n">
+        <v>2780.2</v>
       </c>
     </row>
   </sheetData>
@@ -4444,19 +4457,19 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>17.928054</v>
+        <v>151.757746</v>
       </c>
       <c r="C105" t="n">
-        <v>29.770021</v>
+        <v>450.038294</v>
       </c>
       <c r="D105" t="n">
-        <v>44.383431</v>
+        <v>646.796545</v>
       </c>
       <c r="E105" t="n">
-        <v>15.288094</v>
+        <v>331.174542</v>
       </c>
       <c r="F105" t="n">
-        <v>64.80995799999999</v>
+        <v>873.277272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: full precision for 2026 Q2 consumption data
Q2 sheet in the downloadable Excel was re-deriving from the chart's
1-decimal-rounded CONSUM_VALUES array, losing precision below ~100 MWh.
Backfilled Jan-Aug 2026 with unrounded totals from the raw ARCONEL file,
and the update script now keeps 3 decimal places (MWh-level) going forward.
</commit_message>
<xml_diff>
--- a/electricidad/facturacion_clientes_regulados_resumen.xlsx
+++ b/electricidad/facturacion_clientes_regulados_resumen.xlsx
@@ -1901,7 +1901,7 @@
         <v>2566.3</v>
       </c>
       <c r="C87" t="n">
-        <v>2636.5</v>
+        <v>2636.4</v>
       </c>
     </row>
     <row r="88">
@@ -1979,7 +1979,7 @@
         <v>2592.2</v>
       </c>
       <c r="C93" t="n">
-        <v>2684.4</v>
+        <v>2684.3</v>
       </c>
     </row>
     <row r="94">
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>2685.6</v>
+        <v>2685.556</v>
       </c>
       <c r="C98" t="n">
         <v>2724.3</v>
@@ -2054,10 +2054,10 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>2609.1</v>
+        <v>2609.136</v>
       </c>
       <c r="C99" t="n">
-        <v>2732.3</v>
+        <v>2732.2</v>
       </c>
     </row>
     <row r="100">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>3010.2</v>
+        <v>3010.231</v>
       </c>
       <c r="C100" t="n">
         <v>2740.2</v>
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>2911.6</v>
+        <v>2911.556</v>
       </c>
       <c r="C101" t="n">
         <v>2748.2</v>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>3074.6</v>
+        <v>3074.554</v>
       </c>
       <c r="C102" t="n">
         <v>2756.2</v>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>3040.6</v>
+        <v>3040.645</v>
       </c>
       <c r="C103" t="n">
         <v>2764.2</v>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>3208.7</v>
+        <v>3208.656</v>
       </c>
       <c r="C104" t="n">
         <v>2772.2</v>
@@ -2132,10 +2132,10 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>3058.6</v>
+        <v>3058.61</v>
       </c>
       <c r="C105" t="n">
-        <v>2780.2</v>
+        <v>2780.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>